<commit_message>
Refactor code structure and remove redundant changes
</commit_message>
<xml_diff>
--- a/paper/data/merapi_liq.xlsx
+++ b/paper/data/merapi_liq.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B07AC94-A2DD-4105-B42D-4E3D14371270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99394154-AFC7-4513-8EDA-697C2640E311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3470" yWindow="3080" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14920" yWindow="9350" windowWidth="23300" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1910,7 +1910,9 @@
       <c r="P25" s="7">
         <v>0.26</v>
       </c>
-      <c r="Q25" s="7"/>
+      <c r="Q25" s="7">
+        <v>100.21</v>
+      </c>
       <c r="S25" s="5"/>
       <c r="T25" s="3"/>
       <c r="V25" s="3"/>
@@ -1970,7 +1972,9 @@
       <c r="P26" s="7">
         <v>0.28999999999999998</v>
       </c>
-      <c r="Q26" s="7"/>
+      <c r="Q26" s="7">
+        <v>100.36</v>
+      </c>
       <c r="S26" s="5"/>
       <c r="T26" s="3"/>
       <c r="V26" s="3"/>
@@ -2030,7 +2034,9 @@
       <c r="P27" s="7">
         <v>0.31</v>
       </c>
-      <c r="Q27" s="7"/>
+      <c r="Q27" s="7">
+        <v>99.91</v>
+      </c>
       <c r="T27" s="3"/>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.35">
@@ -2078,7 +2084,9 @@
       <c r="P28" s="7">
         <v>0.28999999999999998</v>
       </c>
-      <c r="Q28" s="7"/>
+      <c r="Q28" s="7">
+        <v>99.93</v>
+      </c>
       <c r="T28" s="3"/>
     </row>
   </sheetData>

</xml_diff>